<commit_message>
Correct the classification time recorded in S5_outcome_level.csv
The classified_at value was entered from a wrong clock reading; it is now the
time the file was written (2026-10-26T20:07Z). Readable copies regenerated.
</commit_message>
<xml_diff>
--- a/S5/S5_placement_data.xlsx
+++ b/S5/S5_placement_data.xlsx
@@ -31086,7 +31086,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31118,7 +31118,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31150,7 +31150,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31182,7 +31182,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31214,7 +31214,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31246,7 +31246,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31278,7 +31278,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31310,7 +31310,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31342,7 +31342,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31374,7 +31374,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31406,7 +31406,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31438,7 +31438,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31470,7 +31470,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31502,7 +31502,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31534,7 +31534,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31566,7 +31566,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31598,7 +31598,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31630,7 +31630,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31662,7 +31662,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31694,7 +31694,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31726,7 +31726,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31758,7 +31758,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31790,7 +31790,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31822,7 +31822,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31854,7 +31854,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31886,7 +31886,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31918,7 +31918,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31950,7 +31950,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -31982,7 +31982,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>
@@ -32014,7 +32014,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-10-26T23:10Z</t>
+          <t>2026-10-26T20:07Z</t>
         </is>
       </c>
     </row>

</xml_diff>